<commit_message>
결과 파일 업데이트 2026-08-07 10:00
</commit_message>
<xml_diff>
--- a/results/andar_할인율모니터링_20260807.xlsx
+++ b/results/andar_할인율모니터링_20260807.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H178"/>
+  <dimension ref="A1:H175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,7 +491,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>9,911</t>
+          <t>9,912</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>245</t>
+          <t>247</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -617,7 +617,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>245</t>
+          <t>247</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -659,7 +659,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>245</t>
+          <t>247</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>3,367</t>
+          <t>3,368</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>3,367</t>
+          <t>3,368</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -911,7 +911,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>7,109</t>
+          <t>7,113</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -995,7 +995,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2,141</t>
+          <t>2,143</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1069,17 +1069,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>32,000</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>17%</t>
+          <t>9%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>1,064</t>
+          <t>1,065</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1237,12 +1237,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>37,000</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>26%</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1373,7 +1373,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>301</t>
+          <t>302</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1457,7 +1457,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>89</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>310</t>
+          <t>311</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1625,7 +1625,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>4,926</t>
+          <t>4,927</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1793,7 +1793,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>1,003</t>
+          <t>1,005</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>1,003</t>
+          <t>1,005</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>680</t>
+          <t>681</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>1,919</t>
+          <t>1,920</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -6035,7 +6035,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>1,919</t>
+          <t>1,920</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
@@ -7601,37 +7601,37 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11375&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10489&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>ENTSC-03</t>
+          <t>EMTRI-02</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>[3 SET] 에어프레시 페이크 삭스</t>
+          <t>서스테이너블 뉴웨이브 요가링</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>19,000</t>
+          <t>33,000</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>58%</t>
+          <t>15%</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>640</t>
+          <t>151</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
@@ -7643,37 +7643,37 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11374&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10191&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>ENTSC-04</t>
+          <t>EMTSC-26</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>[7 SET] 에어프레시 페이크 삭스</t>
+          <t>[1&amp;1] 램스울 크루 삭스</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>105,000</t>
+          <t>19,800</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>17,900</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>63%</t>
+          <t>10%</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>640</t>
+          <t>743</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
@@ -7685,208 +7685,82 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11373&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12511&amp;cate_no=2111&amp;display_group=1</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>ENTSC-02</t>
+          <t>ENTSO-03</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>에어프레시 페이크 삭스</t>
+          <t>안다르 이지무브 화이트</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>15,000</t>
+          <t>129,000</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>64,500</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>34%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>640</t>
+          <t>491</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.5</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10489&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12512&amp;cate_no=2111&amp;display_group=1</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>EMTRI-02</t>
+          <t>ENTSO-03</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>서스테이너블 뉴웨이브 요가링</t>
+          <t>안다르 이지무브 베이지</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>129,000</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>33,000</t>
+          <t>64,500</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>151</t>
+          <t>410</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
-        <is>
-          <t>4.8</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10191&amp;cate_no=2100&amp;display_group=1</t>
-        </is>
-      </c>
-      <c r="B176" t="inlineStr">
-        <is>
-          <t>EMTSC-26</t>
-        </is>
-      </c>
-      <c r="C176" t="inlineStr">
-        <is>
-          <t>[1&amp;1] 램스울 크루 삭스</t>
-        </is>
-      </c>
-      <c r="D176" t="inlineStr">
-        <is>
-          <t>19,800</t>
-        </is>
-      </c>
-      <c r="E176" t="inlineStr">
-        <is>
-          <t>17,900</t>
-        </is>
-      </c>
-      <c r="F176" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="G176" t="inlineStr">
-        <is>
-          <t>743</t>
-        </is>
-      </c>
-      <c r="H176" t="inlineStr">
-        <is>
-          <t>4.8</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="inlineStr">
-        <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12511&amp;cate_no=2111&amp;display_group=1</t>
-        </is>
-      </c>
-      <c r="B177" t="inlineStr">
-        <is>
-          <t>ENTSO-03</t>
-        </is>
-      </c>
-      <c r="C177" t="inlineStr">
-        <is>
-          <t>안다르 이지무브 화이트</t>
-        </is>
-      </c>
-      <c r="D177" t="inlineStr">
-        <is>
-          <t>129,000</t>
-        </is>
-      </c>
-      <c r="E177" t="inlineStr">
-        <is>
-          <t>64,500</t>
-        </is>
-      </c>
-      <c r="F177" t="inlineStr">
-        <is>
-          <t>50%</t>
-        </is>
-      </c>
-      <c r="G177" t="inlineStr">
-        <is>
-          <t>491</t>
-        </is>
-      </c>
-      <c r="H177" t="inlineStr">
-        <is>
-          <t>4.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12512&amp;cate_no=2111&amp;display_group=1</t>
-        </is>
-      </c>
-      <c r="B178" t="inlineStr">
-        <is>
-          <t>ENTSO-03</t>
-        </is>
-      </c>
-      <c r="C178" t="inlineStr">
-        <is>
-          <t>안다르 이지무브 베이지</t>
-        </is>
-      </c>
-      <c r="D178" t="inlineStr">
-        <is>
-          <t>129,000</t>
-        </is>
-      </c>
-      <c r="E178" t="inlineStr">
-        <is>
-          <t>64,500</t>
-        </is>
-      </c>
-      <c r="F178" t="inlineStr">
-        <is>
-          <t>50%</t>
-        </is>
-      </c>
-      <c r="G178" t="inlineStr">
-        <is>
-          <t>410</t>
-        </is>
-      </c>
-      <c r="H178" t="inlineStr">
         <is>
           <t>4.6</t>
         </is>

</xml_diff>